<commit_message>
Update for week of Fri. July 03 26
</commit_message>
<xml_diff>
--- a/FORGE_INFO698_Gantt.xlsx
+++ b/FORGE_INFO698_Gantt.xlsx
@@ -599,7 +599,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-03</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F16" s="10" t="n"/>

</xml_diff>

<commit_message>
week 7 and 8
</commit_message>
<xml_diff>
--- a/FORGE_INFO698_Gantt.xlsx
+++ b/FORGE_INFO698_Gantt.xlsx
@@ -599,7 +599,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-16</t>
         </is>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>done</t>
         </is>
       </c>
       <c r="F19" s="10" t="n"/>
@@ -1182,7 +1182,7 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>done</t>
         </is>
       </c>
       <c r="F20" s="10" t="n"/>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F21" s="10" t="n"/>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F22" s="10" t="n"/>

</xml_diff>

<commit_message>
Added final signed proposal + pane for it
</commit_message>
<xml_diff>
--- a/FORGE_INFO698_Gantt.xlsx
+++ b/FORGE_INFO698_Gantt.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R52"/>
+  <dimension ref="A1:R58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -599,7 +599,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-07</t>
         </is>
       </c>
     </row>
@@ -728,7 +728,7 @@
       <c r="N7" s="11" t="n"/>
       <c r="O7" s="11" t="n"/>
       <c r="P7" s="11" t="n"/>
-      <c r="Q7" s="10" t="n"/>
+      <c r="Q7" s="11" t="n"/>
       <c r="R7" s="10" t="n"/>
     </row>
     <row r="8">
@@ -764,7 +764,7 @@
       <c r="N8" s="11" t="n"/>
       <c r="O8" s="11" t="n"/>
       <c r="P8" s="11" t="n"/>
-      <c r="Q8" s="10" t="n"/>
+      <c r="Q8" s="11" t="n"/>
       <c r="R8" s="10" t="n"/>
     </row>
     <row r="9">
@@ -800,7 +800,7 @@
       <c r="N9" s="11" t="n"/>
       <c r="O9" s="11" t="n"/>
       <c r="P9" s="11" t="n"/>
-      <c r="Q9" s="10" t="n"/>
+      <c r="Q9" s="11" t="n"/>
       <c r="R9" s="10" t="n"/>
     </row>
     <row r="10">
@@ -836,7 +836,7 @@
       <c r="N10" s="11" t="n"/>
       <c r="O10" s="11" t="n"/>
       <c r="P10" s="11" t="n"/>
-      <c r="Q10" s="10" t="n"/>
+      <c r="Q10" s="11" t="n"/>
       <c r="R10" s="10" t="n"/>
     </row>
     <row r="11">
@@ -872,7 +872,7 @@
       <c r="N11" s="11" t="n"/>
       <c r="O11" s="11" t="n"/>
       <c r="P11" s="11" t="n"/>
-      <c r="Q11" s="10" t="n"/>
+      <c r="Q11" s="11" t="n"/>
       <c r="R11" s="10" t="n"/>
     </row>
     <row r="12">
@@ -908,7 +908,7 @@
       <c r="N12" s="11" t="n"/>
       <c r="O12" s="11" t="n"/>
       <c r="P12" s="11" t="n"/>
-      <c r="Q12" s="10" t="n"/>
+      <c r="Q12" s="11" t="n"/>
       <c r="R12" s="10" t="n"/>
     </row>
     <row r="13">
@@ -944,7 +944,7 @@
       <c r="N13" s="11" t="n"/>
       <c r="O13" s="11" t="n"/>
       <c r="P13" s="11" t="n"/>
-      <c r="Q13" s="10" t="n"/>
+      <c r="Q13" s="11" t="n"/>
       <c r="R13" s="10" t="n"/>
     </row>
     <row r="14">
@@ -980,7 +980,7 @@
       <c r="N14" s="11" t="n"/>
       <c r="O14" s="11" t="n"/>
       <c r="P14" s="11" t="n"/>
-      <c r="Q14" s="10" t="n"/>
+      <c r="Q14" s="11" t="n"/>
       <c r="R14" s="10" t="n"/>
     </row>
     <row r="15">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>done</t>
         </is>
       </c>
       <c r="F15" s="10" t="n"/>
@@ -1016,7 +1016,7 @@
       <c r="N15" s="11" t="n"/>
       <c r="O15" s="11" t="n"/>
       <c r="P15" s="11" t="n"/>
-      <c r="Q15" s="10" t="n"/>
+      <c r="Q15" s="11" t="n"/>
       <c r="R15" s="10" t="n"/>
     </row>
     <row r="16">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>done</t>
         </is>
       </c>
       <c r="F16" s="10" t="n"/>
@@ -1052,7 +1052,7 @@
       <c r="N16" s="11" t="n"/>
       <c r="O16" s="11" t="n"/>
       <c r="P16" s="11" t="n"/>
-      <c r="Q16" s="10" t="n"/>
+      <c r="Q16" s="11" t="n"/>
       <c r="R16" s="10" t="n"/>
     </row>
     <row r="17">
@@ -1070,11 +1070,11 @@
         <v>46188</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>46208</v>
+        <v>46243</v>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>done</t>
         </is>
       </c>
       <c r="F17" s="10" t="n"/>
@@ -1084,11 +1084,11 @@
       <c r="J17" s="12" t="n"/>
       <c r="K17" s="12" t="n"/>
       <c r="L17" s="12" t="n"/>
-      <c r="M17" s="10" t="n"/>
-      <c r="N17" s="11" t="n"/>
-      <c r="O17" s="11" t="n"/>
-      <c r="P17" s="11" t="n"/>
-      <c r="Q17" s="10" t="n"/>
+      <c r="M17" s="12" t="n"/>
+      <c r="N17" s="12" t="n"/>
+      <c r="O17" s="12" t="n"/>
+      <c r="P17" s="12" t="n"/>
+      <c r="Q17" s="12" t="n"/>
       <c r="R17" s="10" t="n"/>
     </row>
     <row r="18">
@@ -1106,11 +1106,11 @@
         <v>46188</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>46208</v>
+        <v>46243</v>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>done</t>
         </is>
       </c>
       <c r="F18" s="10" t="n"/>
@@ -1120,29 +1120,29 @@
       <c r="J18" s="12" t="n"/>
       <c r="K18" s="12" t="n"/>
       <c r="L18" s="12" t="n"/>
-      <c r="M18" s="10" t="n"/>
-      <c r="N18" s="11" t="n"/>
-      <c r="O18" s="11" t="n"/>
-      <c r="P18" s="11" t="n"/>
-      <c r="Q18" s="10" t="n"/>
+      <c r="M18" s="12" t="n"/>
+      <c r="N18" s="12" t="n"/>
+      <c r="O18" s="12" t="n"/>
+      <c r="P18" s="12" t="n"/>
+      <c r="Q18" s="12" t="n"/>
       <c r="R18" s="10" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>MVP — Phase 2 (integrate + deploy)</t>
+          <t>MVP — Phase 1 (standalone)</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Integrate repos → FORGE website</t>
+          <t>Phonon mk4 — Bayesian head + Pareto frontier</t>
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>46209</v>
+        <v>46230</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>46222</v>
+        <v>46243</v>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
@@ -1156,29 +1156,29 @@
       <c r="J19" s="10" t="n"/>
       <c r="K19" s="10" t="n"/>
       <c r="L19" s="10" t="n"/>
-      <c r="M19" s="13" t="n"/>
-      <c r="N19" s="13" t="n"/>
+      <c r="M19" s="10" t="n"/>
+      <c r="N19" s="11" t="n"/>
       <c r="O19" s="11" t="n"/>
-      <c r="P19" s="11" t="n"/>
-      <c r="Q19" s="10" t="n"/>
+      <c r="P19" s="12" t="n"/>
+      <c r="Q19" s="12" t="n"/>
       <c r="R19" s="10" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>MVP — Phase 2 (integrate + deploy)</t>
+          <t>MVP — Phase 1 (standalone)</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Deploy: localhost → external hosting</t>
+          <t>ATLAS LLP — three rungs + DNCn_QN closure</t>
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>46209</v>
+        <v>46237</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>46222</v>
+        <v>46243</v>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
@@ -1192,11 +1192,11 @@
       <c r="J20" s="10" t="n"/>
       <c r="K20" s="10" t="n"/>
       <c r="L20" s="10" t="n"/>
-      <c r="M20" s="13" t="n"/>
-      <c r="N20" s="13" t="n"/>
+      <c r="M20" s="10" t="n"/>
+      <c r="N20" s="11" t="n"/>
       <c r="O20" s="11" t="n"/>
       <c r="P20" s="11" t="n"/>
-      <c r="Q20" s="10" t="n"/>
+      <c r="Q20" s="12" t="n"/>
       <c r="R20" s="10" t="n"/>
     </row>
     <row r="21">
@@ -1207,14 +1207,14 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Finalize Bayesian / dashboard decisions</t>
+          <t>Integrate repos → FORGE website</t>
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>46216</v>
+        <v>46209</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>46229</v>
+        <v>46222</v>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
@@ -1228,11 +1228,11 @@
       <c r="J21" s="10" t="n"/>
       <c r="K21" s="10" t="n"/>
       <c r="L21" s="10" t="n"/>
-      <c r="M21" s="10" t="n"/>
+      <c r="M21" s="13" t="n"/>
       <c r="N21" s="13" t="n"/>
-      <c r="O21" s="13" t="n"/>
+      <c r="O21" s="11" t="n"/>
       <c r="P21" s="11" t="n"/>
-      <c r="Q21" s="10" t="n"/>
+      <c r="Q21" s="11" t="n"/>
       <c r="R21" s="10" t="n"/>
     </row>
     <row r="22">
@@ -1243,14 +1243,14 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>FORGE contract + gauge lock-in</t>
+          <t>Deploy: localhost → external hosting</t>
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>46223</v>
+        <v>46209</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>46229</v>
+        <v>46222</v>
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
@@ -1264,11 +1264,11 @@
       <c r="J22" s="10" t="n"/>
       <c r="K22" s="10" t="n"/>
       <c r="L22" s="10" t="n"/>
-      <c r="M22" s="10" t="n"/>
-      <c r="N22" s="11" t="n"/>
-      <c r="O22" s="13" t="n"/>
+      <c r="M22" s="13" t="n"/>
+      <c r="N22" s="13" t="n"/>
+      <c r="O22" s="11" t="n"/>
       <c r="P22" s="11" t="n"/>
-      <c r="Q22" s="10" t="n"/>
+      <c r="Q22" s="11" t="n"/>
       <c r="R22" s="10" t="n"/>
     </row>
     <row r="23">
@@ -1279,18 +1279,18 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Front-end design restart (FORGE_site_dev)</t>
+          <t>Finalize Bayesian / dashboard decisions</t>
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>46223</v>
+        <v>46216</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>46236</v>
+        <v>46229</v>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>done</t>
         </is>
       </c>
       <c r="F23" s="10" t="n"/>
@@ -1301,10 +1301,10 @@
       <c r="K23" s="10" t="n"/>
       <c r="L23" s="10" t="n"/>
       <c r="M23" s="10" t="n"/>
-      <c r="N23" s="11" t="n"/>
+      <c r="N23" s="13" t="n"/>
       <c r="O23" s="13" t="n"/>
-      <c r="P23" s="13" t="n"/>
-      <c r="Q23" s="10" t="n"/>
+      <c r="P23" s="11" t="n"/>
+      <c r="Q23" s="11" t="n"/>
       <c r="R23" s="10" t="n"/>
     </row>
     <row r="24">
@@ -1315,18 +1315,18 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Tutorial example — Palmer Penguins (forge-lite)</t>
+          <t>FORGE contract + gauge lock-in</t>
         </is>
       </c>
       <c r="C24" s="7" t="n">
         <v>46223</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>46236</v>
+        <v>46229</v>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>done</t>
         </is>
       </c>
       <c r="F24" s="10" t="n"/>
@@ -1339,8 +1339,8 @@
       <c r="M24" s="10" t="n"/>
       <c r="N24" s="11" t="n"/>
       <c r="O24" s="13" t="n"/>
-      <c r="P24" s="13" t="n"/>
-      <c r="Q24" s="10" t="n"/>
+      <c r="P24" s="11" t="n"/>
+      <c r="Q24" s="11" t="n"/>
       <c r="R24" s="10" t="n"/>
     </row>
     <row r="25">
@@ -1351,14 +1351,14 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>FORGE hype video</t>
+          <t>Front-end design restart (FORGE_site_dev)</t>
         </is>
       </c>
       <c r="C25" s="7" t="n">
         <v>46223</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>46229</v>
+        <v>46236</v>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
@@ -1375,8 +1375,8 @@
       <c r="M25" s="10" t="n"/>
       <c r="N25" s="11" t="n"/>
       <c r="O25" s="13" t="n"/>
-      <c r="P25" s="11" t="n"/>
-      <c r="Q25" s="10" t="n"/>
+      <c r="P25" s="13" t="n"/>
+      <c r="Q25" s="11" t="n"/>
       <c r="R25" s="10" t="n"/>
     </row>
     <row r="26">
@@ -1387,18 +1387,18 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Test &amp; debug integrated stack</t>
+          <t>Tutorial example — penguins → Brandeis dice</t>
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>46209</v>
+        <v>46223</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>46229</v>
+        <v>46243</v>
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>done</t>
         </is>
       </c>
       <c r="F26" s="10" t="n"/>
@@ -1408,11 +1408,11 @@
       <c r="J26" s="10" t="n"/>
       <c r="K26" s="10" t="n"/>
       <c r="L26" s="10" t="n"/>
-      <c r="M26" s="13" t="n"/>
-      <c r="N26" s="13" t="n"/>
+      <c r="M26" s="10" t="n"/>
+      <c r="N26" s="11" t="n"/>
       <c r="O26" s="13" t="n"/>
-      <c r="P26" s="11" t="n"/>
-      <c r="Q26" s="10" t="n"/>
+      <c r="P26" s="13" t="n"/>
+      <c r="Q26" s="13" t="n"/>
       <c r="R26" s="10" t="n"/>
     </row>
     <row r="27">
@@ -1423,18 +1423,18 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Final software edits + testing</t>
+          <t>FORGE hype video</t>
         </is>
       </c>
       <c r="C27" s="7" t="n">
         <v>46223</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>46236</v>
+        <v>46229</v>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>in_progress</t>
+          <t>done</t>
         </is>
       </c>
       <c r="F27" s="10" t="n"/>
@@ -1447,8 +1447,8 @@
       <c r="M27" s="10" t="n"/>
       <c r="N27" s="11" t="n"/>
       <c r="O27" s="13" t="n"/>
-      <c r="P27" s="13" t="n"/>
-      <c r="Q27" s="10" t="n"/>
+      <c r="P27" s="11" t="n"/>
+      <c r="Q27" s="11" t="n"/>
       <c r="R27" s="10" t="n"/>
     </row>
     <row r="28">
@@ -1459,18 +1459,18 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Begin write-up (slipped W9 → W10)</t>
+          <t>Variance base measure + C1–C4 lock-in</t>
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>46230</v>
+        <v>46237</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>46236</v>
+        <v>46243</v>
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>done</t>
         </is>
       </c>
       <c r="F28" s="10" t="n"/>
@@ -1483,30 +1483,30 @@
       <c r="M28" s="10" t="n"/>
       <c r="N28" s="11" t="n"/>
       <c r="O28" s="11" t="n"/>
-      <c r="P28" s="13" t="n"/>
-      <c r="Q28" s="10" t="n"/>
+      <c r="P28" s="11" t="n"/>
+      <c r="Q28" s="13" t="n"/>
       <c r="R28" s="10" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>MVP — Phase 3 / stretch</t>
+          <t>MVP — Phase 2 (integrate + deploy)</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Lock MVP + freeze repos</t>
+          <t>FORGE board export + packaging (8 models)</t>
         </is>
       </c>
       <c r="C29" s="7" t="n">
-        <v>46230</v>
+        <v>46237</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>46236</v>
+        <v>46243</v>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>done</t>
         </is>
       </c>
       <c r="F29" s="10" t="n"/>
@@ -1519,30 +1519,30 @@
       <c r="M29" s="10" t="n"/>
       <c r="N29" s="11" t="n"/>
       <c r="O29" s="11" t="n"/>
-      <c r="P29" s="14" t="n"/>
-      <c r="Q29" s="10" t="n"/>
+      <c r="P29" s="11" t="n"/>
+      <c r="Q29" s="13" t="n"/>
       <c r="R29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>MVP — Phase 3 / stretch</t>
+          <t>MVP — Phase 2 (integrate + deploy)</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Stretch goal (if time)</t>
+          <t>Test &amp; debug integrated stack</t>
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>46230</v>
+        <v>46209</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>46236</v>
+        <v>46243</v>
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F30" s="10" t="n"/>
@@ -1552,33 +1552,33 @@
       <c r="J30" s="10" t="n"/>
       <c r="K30" s="10" t="n"/>
       <c r="L30" s="10" t="n"/>
-      <c r="M30" s="10" t="n"/>
-      <c r="N30" s="11" t="n"/>
-      <c r="O30" s="11" t="n"/>
-      <c r="P30" s="14" t="n"/>
-      <c r="Q30" s="10" t="n"/>
+      <c r="M30" s="13" t="n"/>
+      <c r="N30" s="13" t="n"/>
+      <c r="O30" s="13" t="n"/>
+      <c r="P30" s="13" t="n"/>
+      <c r="Q30" s="13" t="n"/>
       <c r="R30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Write-up / Deliverables</t>
+          <t>MVP — Phase 2 (integrate + deploy)</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Finish write-up; deliverables locked</t>
+          <t>Final software edits + testing</t>
         </is>
       </c>
       <c r="C31" s="7" t="n">
-        <v>46237</v>
+        <v>46223</v>
       </c>
       <c r="D31" s="7" t="n">
         <v>46243</v>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F31" s="10" t="n"/>
@@ -1590,31 +1590,31 @@
       <c r="L31" s="10" t="n"/>
       <c r="M31" s="10" t="n"/>
       <c r="N31" s="11" t="n"/>
-      <c r="O31" s="11" t="n"/>
-      <c r="P31" s="11" t="n"/>
-      <c r="Q31" s="15" t="n"/>
+      <c r="O31" s="13" t="n"/>
+      <c r="P31" s="13" t="n"/>
+      <c r="Q31" s="13" t="n"/>
       <c r="R31" s="10" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Turn in</t>
+          <t>MVP — Phase 2 (integrate + deploy)</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Turn in · present · showcase</t>
+          <t>Stitch FORGE site — all components integrated</t>
         </is>
       </c>
       <c r="C32" s="7" t="n">
-        <v>46244</v>
+        <v>46237</v>
       </c>
       <c r="D32" s="7" t="n">
         <v>46250</v>
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>in_progress</t>
         </is>
       </c>
       <c r="F32" s="10" t="n"/>
@@ -1628,228 +1628,444 @@
       <c r="N32" s="11" t="n"/>
       <c r="O32" s="11" t="n"/>
       <c r="P32" s="11" t="n"/>
-      <c r="Q32" s="10" t="n"/>
-      <c r="R32" s="16" t="n"/>
+      <c r="Q32" s="13" t="n"/>
+      <c r="R32" s="13" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="17" t="inlineStr"/>
-      <c r="B33" s="18" t="inlineStr">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>MVP — Phase 2 (integrate + deploy)</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Begin write-up (slipped W9 → W10 → W11)</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>46237</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>46243</v>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="n"/>
+      <c r="G33" s="10" t="n"/>
+      <c r="H33" s="10" t="n"/>
+      <c r="I33" s="10" t="n"/>
+      <c r="J33" s="10" t="n"/>
+      <c r="K33" s="10" t="n"/>
+      <c r="L33" s="10" t="n"/>
+      <c r="M33" s="10" t="n"/>
+      <c r="N33" s="11" t="n"/>
+      <c r="O33" s="11" t="n"/>
+      <c r="P33" s="11" t="n"/>
+      <c r="Q33" s="13" t="n"/>
+      <c r="R33" s="10" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>MVP — Phase 3 / stretch</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Lock MVP + freeze repos</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="n">
+        <v>46237</v>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>46250</v>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="F34" s="10" t="n"/>
+      <c r="G34" s="10" t="n"/>
+      <c r="H34" s="10" t="n"/>
+      <c r="I34" s="10" t="n"/>
+      <c r="J34" s="10" t="n"/>
+      <c r="K34" s="10" t="n"/>
+      <c r="L34" s="10" t="n"/>
+      <c r="M34" s="10" t="n"/>
+      <c r="N34" s="11" t="n"/>
+      <c r="O34" s="11" t="n"/>
+      <c r="P34" s="11" t="n"/>
+      <c r="Q34" s="14" t="n"/>
+      <c r="R34" s="14" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>MVP — Phase 3 / stretch</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Stretch goal (if time)</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="n">
+        <v>46237</v>
+      </c>
+      <c r="D35" s="7" t="n">
+        <v>46243</v>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="n"/>
+      <c r="G35" s="10" t="n"/>
+      <c r="H35" s="10" t="n"/>
+      <c r="I35" s="10" t="n"/>
+      <c r="J35" s="10" t="n"/>
+      <c r="K35" s="10" t="n"/>
+      <c r="L35" s="10" t="n"/>
+      <c r="M35" s="10" t="n"/>
+      <c r="N35" s="11" t="n"/>
+      <c r="O35" s="11" t="n"/>
+      <c r="P35" s="11" t="n"/>
+      <c r="Q35" s="14" t="n"/>
+      <c r="R35" s="10" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Write-up / Deliverables</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Finish write-up; deliverables locked</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>46237</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>46250</v>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="F36" s="10" t="n"/>
+      <c r="G36" s="10" t="n"/>
+      <c r="H36" s="10" t="n"/>
+      <c r="I36" s="10" t="n"/>
+      <c r="J36" s="10" t="n"/>
+      <c r="K36" s="10" t="n"/>
+      <c r="L36" s="10" t="n"/>
+      <c r="M36" s="10" t="n"/>
+      <c r="N36" s="11" t="n"/>
+      <c r="O36" s="11" t="n"/>
+      <c r="P36" s="11" t="n"/>
+      <c r="Q36" s="15" t="n"/>
+      <c r="R36" s="15" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Write-up / Deliverables</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Final report — outline → draft → submit</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>46237</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>46250</v>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+      <c r="F37" s="10" t="n"/>
+      <c r="G37" s="10" t="n"/>
+      <c r="H37" s="10" t="n"/>
+      <c r="I37" s="10" t="n"/>
+      <c r="J37" s="10" t="n"/>
+      <c r="K37" s="10" t="n"/>
+      <c r="L37" s="10" t="n"/>
+      <c r="M37" s="10" t="n"/>
+      <c r="N37" s="11" t="n"/>
+      <c r="O37" s="11" t="n"/>
+      <c r="P37" s="11" t="n"/>
+      <c r="Q37" s="15" t="n"/>
+      <c r="R37" s="15" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Turn in</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Turn in · present · showcase</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>46244</v>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>46250</v>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>planned</t>
+        </is>
+      </c>
+      <c r="F38" s="10" t="n"/>
+      <c r="G38" s="10" t="n"/>
+      <c r="H38" s="10" t="n"/>
+      <c r="I38" s="10" t="n"/>
+      <c r="J38" s="10" t="n"/>
+      <c r="K38" s="10" t="n"/>
+      <c r="L38" s="10" t="n"/>
+      <c r="M38" s="10" t="n"/>
+      <c r="N38" s="11" t="n"/>
+      <c r="O38" s="11" t="n"/>
+      <c r="P38" s="11" t="n"/>
+      <c r="Q38" s="11" t="n"/>
+      <c r="R38" s="16" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="inlineStr"/>
+      <c r="B39" s="18" t="inlineStr">
         <is>
           <t>Milestones (◈)</t>
         </is>
       </c>
-      <c r="C33" s="17" t="n"/>
-      <c r="D33" s="17" t="n"/>
-      <c r="E33" s="17" t="n"/>
-      <c r="F33" s="17" t="n"/>
-      <c r="G33" s="17" t="n"/>
-      <c r="H33" s="19" t="inlineStr">
+      <c r="C39" s="17" t="n"/>
+      <c r="D39" s="17" t="n"/>
+      <c r="E39" s="17" t="n"/>
+      <c r="F39" s="17" t="n"/>
+      <c r="G39" s="17" t="n"/>
+      <c r="H39" s="19" t="inlineStr">
         <is>
           <t>◈1</t>
         </is>
       </c>
-      <c r="I33" s="19" t="inlineStr">
+      <c r="I39" s="19" t="inlineStr">
         <is>
           <t>◈2</t>
         </is>
       </c>
-      <c r="J33" s="17" t="n"/>
-      <c r="K33" s="17" t="n"/>
-      <c r="L33" s="19" t="inlineStr">
+      <c r="J39" s="17" t="n"/>
+      <c r="K39" s="17" t="n"/>
+      <c r="L39" s="19" t="inlineStr">
         <is>
           <t>◈3</t>
         </is>
       </c>
-      <c r="M33" s="17" t="n"/>
-      <c r="N33" s="19" t="inlineStr">
+      <c r="M39" s="17" t="n"/>
+      <c r="N39" s="19" t="inlineStr">
         <is>
           <t>◈4</t>
         </is>
       </c>
-      <c r="O33" s="19" t="inlineStr">
+      <c r="O39" s="19" t="inlineStr">
         <is>
           <t>◈5</t>
         </is>
       </c>
-      <c r="P33" s="19" t="inlineStr">
+      <c r="P39" s="19" t="inlineStr">
         <is>
           <t>◈6</t>
         </is>
       </c>
-      <c r="Q33" s="19" t="inlineStr">
+      <c r="Q39" s="19" t="inlineStr">
         <is>
           <t>◈7</t>
         </is>
       </c>
-      <c r="R33" s="19" t="inlineStr">
+      <c r="R39" s="19" t="inlineStr">
         <is>
           <t>◈8</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
         <is>
           <t>Phase legend</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="9" t="inlineStr"/>
-      <c r="B36" s="4" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr"/>
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>Intro / Planning</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="12" t="inlineStr"/>
-      <c r="B37" s="4" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr"/>
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>MVP — Phase 1 (standalone)</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="13" t="inlineStr"/>
-      <c r="B38" s="4" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr"/>
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>MVP — Phase 2 (integrate + deploy)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="14" t="inlineStr"/>
-      <c r="B39" s="4" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr"/>
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>MVP — Phase 3 / stretch</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="15" t="inlineStr"/>
-      <c r="B40" s="4" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr"/>
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>Write-up / Deliverables</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="16" t="inlineStr"/>
-      <c r="B41" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr"/>
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>Turn in</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="11" t="inlineStr"/>
-      <c r="B42" s="4" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr"/>
+      <c r="B48" s="4" t="inlineStr">
         <is>
           <t>Risk-management window</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="1" t="inlineStr">
-        <is>
-          <t>Milestones</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="1" t="inlineStr">
-        <is>
-          <t>◈1</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>W2 — Proposal mk_1 submitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="1" t="inlineStr">
-        <is>
-          <t>◈2</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>W3 — Full proposal + timeline/Gantt locked</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="1" t="inlineStr">
-        <is>
-          <t>◈3</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>W6 — All three MVP-P1 sites functional (guaranteed floor)</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="1" t="inlineStr">
-        <is>
-          <t>◈4</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>W8 — Integrated FORGE site deployed (Phase 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="1" t="inlineStr">
-        <is>
-          <t>◈5</t>
-        </is>
-      </c>
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>W9 — Front end restarted (select deck + splash); contract + gauges locked; write-up start → W10</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>◈6</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>W10 — MVP + repos locked</t>
+          <t>Milestones</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>◈7</t>
+          <t>◈1</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>W11 — Write-up complete; deliverables locked</t>
+          <t>W2 — Proposal mk_1 submitted</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
+          <t>◈2</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>W3 — Full proposal + timeline/Gantt locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>◈3</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>W6 — All three MVP-P1 sites functional (guaranteed floor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>◈4</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>W8 — Integrated FORGE site deployed (Phase 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>◈5</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>W9 — Front end restarted (select deck + splash); contract + gauges locked; write-up start → W10</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>◈6</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>W10 — Tutorial re-locked (Brandeis dice); phonon mk4 opened; write-up → W11</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>◈7</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>W11 — Variance lock-in; phonon mk4 + ATLAS LLP closed; FORGE board packaged</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
           <t>◈8</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>W12 — Final hand-in / showcase</t>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>W12 — Site stitched · final report submitted · showcase</t>
         </is>
       </c>
     </row>

</xml_diff>